<commit_message>
Close VERA trade at 43.21 via trailing stop
Stop hit before the 2026-07-07 FDA PDUFA catalyst, banking +1.10R
ahead of the binary event. Filled stop_price (~5% trailing, as
reported) and position_size (EUR 150 default) which were missing
at entry, enabling planned_r/r_multiple computation. followed_plan
and lesson still need user input, flagged pink in the Legend.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -83,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -95,6 +96,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -174,10 +176,21 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
+    <author>Claude</author>
     <author>Journal</author>
   </authors>
   <commentList>
-    <comment ref="L9" authorId="0" shapeId="0">
+    <comment ref="L6" authorId="0" shapeId="0">
+      <text>
+        <t>Approximate: trailing stop ~5% below entry (40.95), as reported at close. Not the exact trail-trigger price, since trailing stops move with price.</t>
+      </text>
+    </comment>
+    <comment ref="N6" authorId="0" shapeId="0">
+      <text>
+        <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase fixed sizing; not recorded at entry. Correct if actual size differed.</t>
+      </text>
+    </comment>
+    <comment ref="L9" authorId="1" shapeId="0">
       <text>
         <t>Stop = entry price. This needs correction — R-multiples can't be computed with zero risk.</t>
       </text>
@@ -980,11 +993,15 @@
       <c r="K6" s="2" t="n">
         <v>40.95</v>
       </c>
-      <c r="L6" s="4" t="n"/>
+      <c r="L6" s="2" t="n">
+        <v>38.9</v>
+      </c>
       <c r="M6" s="2" t="n">
         <v>56.04</v>
       </c>
-      <c r="N6" s="4" t="n"/>
+      <c r="N6" s="2" t="n">
+        <v>150</v>
+      </c>
       <c r="O6" s="4" t="n"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -996,18 +1013,28 @@
           <t>Med</t>
         </is>
       </c>
-      <c r="R6" s="4" t="n"/>
+      <c r="R6" s="2" t="n">
+        <v>7.36</v>
+      </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="T6" s="4" t="n"/>
-      <c r="U6" s="4" t="n"/>
-      <c r="V6" s="4" t="n"/>
-      <c r="W6" s="4" t="n"/>
-      <c r="X6" s="4" t="n"/>
-      <c r="Y6" s="4" t="n"/>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="T6" s="9" t="n">
+        <v>46203</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>43.21</v>
+      </c>
+      <c r="V6" s="2" t="n">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="X6" s="5" t="n"/>
+      <c r="Y6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1408,7 +1435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1451,10 +1478,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -1563,10 +1586,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
-    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -1618,12 +1637,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3 closed trades missing followed_plan + lesson</t>
+          <t>4 closed trades missing followed_plan + lesson</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AYI, FCEL, ALI1.DE — these are the fields that make closing a learning event.</t>
+          <t>AYI, FCEL, ALI1.DE, VERA — these are the fields that make closing a learning event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>VERA stop_price + position_size</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Stop (38.90) is an approximation of a ~5% trailing stop reported at close, not the exact trail price. Position size defaulted to EUR 150 (RISK_RULES.md default) since not recorded at entry.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close AMD at 582.91, fill VERA followed_plan/lesson
AMD: corrected the stop=entry placeholder to a ~5% trailing stop
(466.90), matching the convention used for VERA. r_multiple +3.72R.
VERA: followed_plan=partial, lesson notes the 5% trail may have been
too tight. AMD still needs followed_plan/lesson, flagged pink.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -177,7 +177,6 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Claude</author>
-    <author>Journal</author>
   </authors>
   <commentList>
     <comment ref="L6" authorId="0" shapeId="0">
@@ -190,9 +189,9 @@
         <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase fixed sizing; not recorded at entry. Correct if actual size differed.</t>
       </text>
     </comment>
-    <comment ref="L9" authorId="1" shapeId="0">
+    <comment ref="L9" authorId="0" shapeId="0">
       <text>
-        <t>Stop = entry price. This needs correction — R-multiples can't be computed with zero risk.</t>
+        <t>Corrected: original stop=entry was a logging error. Real stop was ~5% below entry, as reported at close.</t>
       </text>
     </comment>
   </commentList>
@@ -1033,8 +1032,16 @@
       <c r="W6" s="2" t="n">
         <v>1.1</v>
       </c>
-      <c r="X6" s="5" t="n"/>
-      <c r="Y6" s="5" t="n"/>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>5% trailing stop was likely too tight for this setup; got shaken out before the catalyst.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1206,8 +1213,8 @@
       <c r="K9" s="2" t="n">
         <v>491.47</v>
       </c>
-      <c r="L9" s="5" t="n">
-        <v>491.47</v>
+      <c r="L9" s="2" t="n">
+        <v>466.9</v>
       </c>
       <c r="M9" s="4" t="n"/>
       <c r="N9" s="2" t="n">
@@ -1223,15 +1230,23 @@
       <c r="R9" s="4" t="n"/>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="n"/>
-      <c r="U9" s="4" t="n"/>
-      <c r="V9" s="4" t="n"/>
-      <c r="W9" s="4" t="n"/>
-      <c r="X9" s="4" t="n"/>
-      <c r="Y9" s="4" t="n"/>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="T9" s="9" t="n">
+        <v>46203</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>582.91</v>
+      </c>
+      <c r="V9" s="2" t="n">
+        <v>26.61</v>
+      </c>
+      <c r="W9" s="2" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="X9" s="5" t="n"/>
+      <c r="Y9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1435,7 +1450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1601,12 +1616,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AMD stop = entry</t>
+          <t>AMD stop = entry (resolved)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Stop price equals entry (491.47). Correct this — R-multiples need nonzero risk.</t>
+          <t>Was a logging error. Corrected to ~5% trailing stop (466.90) at close, per user.</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1657,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AYI, FCEL, ALI1.DE, VERA — these are the fields that make closing a learning event.</t>
+          <t>AYI, FCEL, ALI1.DE, AMD — VERA now filled (partial / stop may be too tight).</t>
         </is>
       </c>
     </row>
@@ -1655,6 +1670,18 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>Stop (38.90) is an approximation of a ~5% trailing stop reported at close, not the exact trail price. Position size defaulted to EUR 150 (RISK_RULES.md default) since not recorded at entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AMD stop_price</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Stop (466.90) is an approximation of a ~5% trailing stop reported at close, replacing the earlier stop=entry placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log ELF and a second MSM entry
ELF (2026-0012): opened today at 85.00, stop 80.00 (-$5/share), from
the 2026-06-28 research addendum. Catalyst date and EPS speculation
flagged unverified. setup_type/thesis/conviction/risk_rating not yet
given, flagged yellow.

MSM (2026-0013): opened 2026-06-29 at 150.00, stop 142.50 (-5%). This
is a separate real entry from the existing 2026-0001 paper-tracked
row (117.91, opened 6/22) -- both kept, not merged, per append-only
convention.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -97,6 +97,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -192,6 +193,31 @@
     <comment ref="L9" authorId="0" shapeId="0">
       <text>
         <t>Corrected: original stop=entry was a logging error. Real stop was ~5% below entry, as reported at close.</t>
+      </text>
+    </comment>
+    <comment ref="H13" authorId="0" shapeId="0">
+      <text>
+        <t>Unverified: recalled/secondhand date and speculated EPS beat, from user, not primary source. Confirm before sizing up.</t>
+      </text>
+    </comment>
+    <comment ref="N13" authorId="0" shapeId="0">
+      <text>
+        <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase sizing; not stated at logging.</t>
+      </text>
+    </comment>
+    <comment ref="I14" authorId="0" shapeId="0">
+      <text>
+        <t>Carried forward from the original 2026-0001 paper-tracked idea for this ticker (same thesis, executed for real one week later at a higher price). Confirm if this is a different setup.</t>
+      </text>
+    </comment>
+    <comment ref="J14" authorId="0" shapeId="0">
+      <text>
+        <t>Carried forward from 2026-0001 (same underlying idea). Confirm if this real entry is unrelated.</t>
+      </text>
+    </comment>
+    <comment ref="N14" authorId="0" shapeId="0">
+      <text>
+        <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase sizing; not stated at logging.</t>
       </text>
     </comment>
   </commentList>
@@ -487,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:Y14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1437,6 +1463,140 @@
       <c r="X12" s="4" t="n"/>
       <c r="Y12" s="4" t="n"/>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-0012</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ELF</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>e.l.f. Beauty</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Q2 FY earnings; ~$0.69/share EPS beat speculated (unverified)</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>46239</v>
+      </c>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" t="n">
+        <v>85</v>
+      </c>
+      <c r="L13" t="n">
+        <v>80</v>
+      </c>
+      <c r="N13" t="n">
+        <v>150</v>
+      </c>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>routine</t>
+        </is>
+      </c>
+      <c r="Q13" s="7" t="n"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>46202</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MSM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MSC Industrial Direct</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Fiscal Q3 earnings</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>46204</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Breakout to new 52-wk highs into earnings, industrial demand improving</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>150</v>
+      </c>
+      <c r="L14" t="n">
+        <v>142.5</v>
+      </c>
+      <c r="N14" t="n">
+        <v>150</v>
+      </c>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>routine</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1450,7 +1610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1685,6 +1845,30 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ELF (2026-0012) missing setup_type/thesis/conviction/risk_rating</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>New real trade from research addendum. Catalyst date and EPS speculation are unverified/recalled, not primary source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>MSM (2026-0013) is a second, separate MSM row</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-0001 (paper, entry 117.91, opened 6/22) is untouched. 2026-0013 is a new real entry at 150, opened 6/29 -- confirm this is the same idea executed later, not a duplicate log.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Correct ELF/MSM entry-vs-position-size mixup, add OPFI
ELF: real entry was 74 (85 was position size). Stop recomputed to
69.00 (-\$5/share). Position size set to 85.

MSM (2026-0013): real entry was 118.95 (150 was position size). Stop
recomputed to 113.00 (-5%). Position size set to 150.

OPFI (2026-0014): new entry at 9.93, found via Finviz + discussed
with Opus, source classified as 'own'. Stop/risk not yet given,
flagged for follow-up.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -200,11 +200,6 @@
         <t>Unverified: recalled/secondhand date and speculated EPS beat, from user, not primary source. Confirm before sizing up.</t>
       </text>
     </comment>
-    <comment ref="N13" authorId="0" shapeId="0">
-      <text>
-        <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase sizing; not stated at logging.</t>
-      </text>
-    </comment>
     <comment ref="I14" authorId="0" shapeId="0">
       <text>
         <t>Carried forward from the original 2026-0001 paper-tracked idea for this ticker (same thesis, executed for real one week later at a higher price). Confirm if this is a different setup.</t>
@@ -215,9 +210,19 @@
         <t>Carried forward from 2026-0001 (same underlying idea). Confirm if this real entry is unrelated.</t>
       </text>
     </comment>
-    <comment ref="N14" authorId="0" shapeId="0">
+    <comment ref="L15" authorId="0" shapeId="0">
+      <text>
+        <t>Not given yet - needed to compute planned_r/r_multiple.</t>
+      </text>
+    </comment>
+    <comment ref="N15" authorId="0" shapeId="0">
       <text>
         <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase sizing; not stated at logging.</t>
+      </text>
+    </comment>
+    <comment ref="P15" authorId="0" shapeId="0">
+      <text>
+        <t>Classified as 'own': found manually via Finviz screener and discussed with Opus, not from the automated scanner pipeline or the weekly research routine. Correct if this should be 'scanner'.</t>
       </text>
     </comment>
   </commentList>
@@ -513,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:Y15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1503,13 +1508,13 @@
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
       <c r="K13" t="n">
+        <v>74</v>
+      </c>
+      <c r="L13" t="n">
+        <v>69</v>
+      </c>
+      <c r="N13" t="n">
         <v>85</v>
-      </c>
-      <c r="L13" t="n">
-        <v>80</v>
-      </c>
-      <c r="N13" t="n">
-        <v>150</v>
       </c>
       <c r="O13" s="7" t="n"/>
       <c r="P13" t="inlineStr">
@@ -1572,10 +1577,10 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>150</v>
+        <v>118.95</v>
       </c>
       <c r="L14" t="n">
-        <v>142.5</v>
+        <v>113</v>
       </c>
       <c r="N14" t="n">
         <v>150</v>
@@ -1592,6 +1597,63 @@
         </is>
       </c>
       <c r="S14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OPFI</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>OppFi Inc.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Found via Finviz screener; reviewed with Opus (Claude) before entry.</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>9.93</v>
+      </c>
+      <c r="L15" s="7" t="n"/>
+      <c r="N15" t="n">
+        <v>150</v>
+      </c>
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="Q15" s="7" t="n"/>
+      <c r="S15" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1610,7 +1672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1853,7 +1915,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>New real trade from research addendum. Catalyst date and EPS speculation are unverified/recalled, not primary source.</t>
+          <t>Real trade from research addendum. Entry 74, stop 69 (-$5), size EUR 85. Catalyst date and EPS speculation unverified/recalled.</t>
         </is>
       </c>
     </row>
@@ -1866,6 +1928,18 @@
       <c r="B23" t="inlineStr">
         <is>
           <t>2026-0001 (paper, entry 117.91, opened 6/22) is untouched. 2026-0013 is a new real entry at 150, opened 6/29 -- confirm this is the same idea executed later, not a duplicate log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>OPFI (2026-0014) missing stop_price/catalyst/setup_type/conviction/risk_rating</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Found via Finviz + discussed with Opus. Entry 9.93. Stop/risk not given yet, needed for planned_r/r_multiple. Size defaulted EUR 150.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill OPFI position size and stop
Same as ELF: EUR 85 position size, -\$5 stop (4.93). Note: this is
~50% risk relative to entry (9.93), flagged in the Legend for
confirmation since it's far outside the stop distances used elsewhere.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -208,16 +208,6 @@
     <comment ref="J14" authorId="0" shapeId="0">
       <text>
         <t>Carried forward from 2026-0001 (same underlying idea). Confirm if this real entry is unrelated.</t>
-      </text>
-    </comment>
-    <comment ref="L15" authorId="0" shapeId="0">
-      <text>
-        <t>Not given yet - needed to compute planned_r/r_multiple.</t>
-      </text>
-    </comment>
-    <comment ref="N15" authorId="0" shapeId="0">
-      <text>
-        <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase sizing; not stated at logging.</t>
       </text>
     </comment>
     <comment ref="P15" authorId="0" shapeId="0">
@@ -1642,9 +1632,11 @@
       <c r="K15" t="n">
         <v>9.93</v>
       </c>
-      <c r="L15" s="7" t="n"/>
+      <c r="L15" t="n">
+        <v>4.93</v>
+      </c>
       <c r="N15" t="n">
-        <v>150</v>
+        <v>85</v>
       </c>
       <c r="O15" s="7" t="n"/>
       <c r="P15" t="inlineStr">
@@ -1934,12 +1926,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>OPFI (2026-0014) missing stop_price/catalyst/setup_type/conviction/risk_rating</t>
+          <t>OPFI (2026-0014) stop is 50% of entry</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Found via Finviz + discussed with Opus. Entry 9.93. Stop/risk not given yet, needed for planned_r/r_multiple. Size defaulted EUR 150.</t>
+          <t>Entry 9.93, stop 4.93 (-$5 as stated) = ~50% risk to stop. Confirm this is intentional; catalyst/setup_type/conviction/risk_rating still not given.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CELC catalyst, close ENR.DE and MSM paper trade
CELC: catalyst set to gedatolisib PDUFA (Jul 17, primary date) plus
Q2 earnings window (Aug 12-14), flagged unverified/recalled.

ENR.DE: closed at 165.22. r_multiple +0.99R, pnl +EUR 8.31.
followed_plan/lesson still needed, flagged pink.

MSM (2026-0001, paper): stopped out at 117.08. No stop was logged at
entry, backfilled as = exit price (exact stop-out, -1.00R). User's
lesson recorded: stop was too tight, shaken out on a sub-5% dip.
followed_plan still needed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -180,6 +180,21 @@
     <author>Claude</author>
   </authors>
   <commentList>
+    <comment ref="L2" authorId="0" shapeId="0">
+      <text>
+        <t>No stop was logged at entry. Backfilled as = exit price (exact stop-out), giving r_multiple = -1.00R by definition.</t>
+      </text>
+    </comment>
+    <comment ref="N2" authorId="0" shapeId="0">
+      <text>
+        <t>Defaulted to EUR 150 per RISK_RULES.md learning-phase sizing; not recorded at entry.</t>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0">
+      <text>
+        <t>Unverified: recalled/secondhand date, not from a primary source (FDA/company IR). Confirm before sizing. Secondary date (Q2 earnings) is Aug 12-14, not separately tracked in this single-date field.</t>
+      </text>
+    </comment>
     <comment ref="L6" authorId="0" shapeId="0">
       <text>
         <t>Approximate: trailing stop ~5% below entry (40.95), as reported at close. Not the exact trail-trigger price, since trailing stops move with price.</t>
@@ -715,9 +730,13 @@
       <c r="K2" s="2" t="n">
         <v>117.91</v>
       </c>
-      <c r="L2" s="4" t="n"/>
+      <c r="L2" s="2" t="n">
+        <v>117.08</v>
+      </c>
       <c r="M2" s="4" t="n"/>
-      <c r="N2" s="4" t="n"/>
+      <c r="N2" s="2" t="n">
+        <v>150</v>
+      </c>
       <c r="O2" s="4" t="n"/>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -732,15 +751,27 @@
       <c r="R2" s="4" t="n"/>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="T2" s="4" t="n"/>
-      <c r="U2" s="4" t="n"/>
-      <c r="V2" s="4" t="n"/>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="T2" s="9" t="n">
+        <v>46203</v>
+      </c>
+      <c r="U2" s="2" t="n">
+        <v>117.08</v>
+      </c>
+      <c r="V2" s="2" t="n">
+        <v>-1.06</v>
+      </c>
+      <c r="W2" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X2" s="5" t="n"/>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>Stop was too tight -- shaken out on a shallow pullback, less than a 5% move. Use a wider stop so a short-term dip does not hurt.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -933,8 +964,14 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA date for gedatolisib (Jul 17); Q2 financial earnings and business update expected Aug 12-14</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>46220</v>
+      </c>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="2" t="n">
@@ -1385,15 +1422,23 @@
       <c r="R11" s="4" t="n"/>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="T11" s="4" t="n"/>
-      <c r="U11" s="4" t="n"/>
-      <c r="V11" s="4" t="n"/>
-      <c r="W11" s="4" t="n"/>
-      <c r="X11" s="4" t="n"/>
-      <c r="Y11" s="4" t="n"/>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="T11" s="9" t="n">
+        <v>46203</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>165.22</v>
+      </c>
+      <c r="V11" s="2" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="W11" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1664,7 +1709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1866,12 +1911,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4 closed trades missing followed_plan + lesson</t>
+          <t>5 closed trades missing followed_plan + lesson</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AYI, FCEL, ALI1.DE, AMD — VERA now filled (partial / stop may be too tight).</t>
+          <t>AYI, FCEL, ALI1.DE, AMD, ENR.DE -- MSM(2026-0001) lesson now filled, followed_plan still open.</t>
         </is>
       </c>
     </row>
@@ -1932,6 +1977,30 @@
       <c r="B24" t="inlineStr">
         <is>
           <t>Entry 9.93, stop 4.93 (-$5 as stated) = ~50% risk to stop. Confirm this is intentional; catalyst/setup_type/conviction/risk_rating still not given.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MSM (2026-0001) stop backfilled at close</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>No stop was set at entry. Backfilled = exit price (117.08), the exact stop-out level, giving -1.00R. Position size defaulted EUR 150.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CELC (2026-0004) catalyst added</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PDUFA Jul 17 (gedatolisib) + Q2 earnings Aug 12-14, unverified/recalled dates. Confirm against a primary source.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add RHM catalyst, log new NBIS trade
RHM: catalyst set to Q2/H1 2026 financial results (Aug 6), flagged
unverified/recalled.

NBIS (2026-0015): limit order filled at 240, trailing 5% stop
(228.00), position size EUR 145. Catalyst/setup_type/thesis/
conviction/risk_rating not yet given, flagged yellow.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -210,6 +210,11 @@
         <t>Corrected: original stop=entry was a logging error. Real stop was ~5% below entry, as reported at close.</t>
       </text>
     </comment>
+    <comment ref="H12" authorId="0" shapeId="0">
+      <text>
+        <t>Unverified: recalled/secondhand date, not from a primary source (company IR/exchange calendar). Confirm before sizing.</t>
+      </text>
+    </comment>
     <comment ref="H13" authorId="0" shapeId="0">
       <text>
         <t>Unverified: recalled/secondhand date and speculated EPS beat, from user, not primary source. Confirm before sizing up.</t>
@@ -228,6 +233,11 @@
     <comment ref="P15" authorId="0" shapeId="0">
       <text>
         <t>Classified as 'own': found manually via Finviz screener and discussed with Opus, not from the automated scanner pipeline or the weekly research routine. Correct if this should be 'scanner'.</t>
+      </text>
+    </comment>
+    <comment ref="L16" authorId="0" shapeId="0">
+      <text>
+        <t>Trailing stop at 5% below entry (240), as stated. Will move with price -- record actual exit level separately at close, same convention as VERA/AMD.</t>
       </text>
     </comment>
   </commentList>
@@ -523,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y15"/>
+  <dimension ref="A1:Y16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1469,8 +1479,14 @@
           <t>Real</t>
         </is>
       </c>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Q2 and H1 2026 financial results</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>46240</v>
+      </c>
       <c r="I12" s="4" t="n"/>
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="2" t="n">
@@ -1691,6 +1707,61 @@
       </c>
       <c r="Q15" s="7" t="n"/>
       <c r="S15" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-0015</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nebius Group</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" t="n">
+        <v>240</v>
+      </c>
+      <c r="L16" t="n">
+        <v>228</v>
+      </c>
+      <c r="N16" t="n">
+        <v>145</v>
+      </c>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="Q16" s="7" t="n"/>
+      <c r="S16" t="inlineStr">
         <is>
           <t>open</t>
         </is>
@@ -1709,7 +1780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2004,6 +2075,30 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RHM (2026-0011) catalyst added</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Q2/H1 2026 financials, Aug 6, unverified/recalled date. Confirm against a primary source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NBIS (2026-0015) missing catalyst/setup_type/thesis/conviction/risk_rating</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Limit order filled at 240, trailing 5% stop (228.00), size EUR 145. Source own.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix corrupted AutoFilter range in journal Excel
The Journal sheet's AutoFilter (and the _xlnm._FilterDatabase defined
name) were stuck at A1:Y12 from an earlier revision, while the sheet
had grown to 16 rows (A1:Y16) after adding ELF/MSM/OPFI/NBIS. That
mismatch between the filter range and actual sheet dimension is a
known Excel corruption trigger (repair-on-open prompt). Extended the
AutoFilter to match the real data range.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zm8rWhJUXuHKVsuCcoddn
</commit_message>
<xml_diff>
--- a/TradingJournalCandidatesTry_updated.xlsx
+++ b/TradingJournalCandidatesTry_updated.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$Y$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Journal'!$A$1:$Y$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1768,7 +1768,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y12"/>
+  <autoFilter ref="A1:Y16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>